<commit_message>
2.4.16: refresh stored figures and Source Data from the independent rerun
</commit_message>
<xml_diff>
--- a/data_derived/figures/source_data/Source_Data_Fig2.xlsx
+++ b/data_derived/figures/source_data/Source_Data_Fig2.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:A5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -458,6 +458,13 @@
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Fig2c_recorded_later: share recorded within each complete horizon, with Wilson intervals simultaneous across the horizons of each release (Bonferroni; formulas).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Counts are database-matched: dates are those of the earliest matching record in the analyzed sources. A literature audit found earlier experimental reports for two of the four OQMD v1.0 compositions recorded within ten years (Supplementary Note 6; marked in Source Data Fig. 1).</t>
         </is>
       </c>
     </row>

</xml_diff>